<commit_message>
load ecoinvent credentials from .env file
</commit_message>
<xml_diff>
--- a/gcam/output/SSP2/iamc_template_gcam_carbon_dioxide_removal.xlsx
+++ b/gcam/output/SSP2/iamc_template_gcam_carbon_dioxide_removal.xlsx
@@ -190,7 +190,7 @@
     <t>Final Energy|Carbon Management|Direct Air Capture|Sorbent</t>
   </si>
   <si>
-    <t>MtC/yr</t>
+    <t>MtCO2/yr</t>
   </si>
   <si>
     <t>EJ/yr</t>
@@ -633,43 +633,43 @@
         <v>58</v>
       </c>
       <c r="H2">
-        <v>0.0002929119</v>
+        <v>0.0010740103</v>
       </c>
       <c r="I2">
-        <v>0.0005472</v>
+        <v>0.0020064</v>
       </c>
       <c r="J2">
-        <v>0.00395988</v>
+        <v>0.01451956</v>
       </c>
       <c r="K2">
-        <v>0.003163074</v>
+        <v>0.011597938</v>
       </c>
       <c r="L2">
-        <v>0.001773732</v>
+        <v>0.006503684</v>
       </c>
       <c r="M2">
-        <v>0.0009285453</v>
+        <v>0.0034046661</v>
       </c>
       <c r="N2">
-        <v>0.000459757</v>
+        <v>0.001685775666666667</v>
       </c>
       <c r="O2">
-        <v>0.0002261763</v>
+        <v>0.0008293131</v>
       </c>
       <c r="P2">
-        <v>0.00010656015</v>
+        <v>0.00039072055</v>
       </c>
       <c r="Q2">
-        <v>5.378237E-05</v>
+        <v>0.0001972020233333333</v>
       </c>
       <c r="R2">
-        <v>2.399709E-05</v>
+        <v>8.798933E-05</v>
       </c>
       <c r="S2">
-        <v>1.270974E-05</v>
+        <v>4.660238E-05</v>
       </c>
       <c r="T2">
-        <v>5.095000000000001E-07</v>
+        <v>1.868166666666667E-06</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -689,43 +689,43 @@
         <v>58</v>
       </c>
       <c r="H3">
-        <v>0.000131175</v>
+        <v>0.000480975</v>
       </c>
       <c r="I3">
-        <v>0.00141985</v>
+        <v>0.005206116666666667</v>
       </c>
       <c r="J3">
-        <v>0.0134002</v>
+        <v>0.04913406666666666</v>
       </c>
       <c r="K3">
-        <v>0.00638373</v>
+        <v>0.02340701</v>
       </c>
       <c r="L3">
-        <v>0.00295743</v>
+        <v>0.01084391</v>
       </c>
       <c r="M3">
-        <v>0.00153487</v>
+        <v>0.005627856666666667</v>
       </c>
       <c r="N3">
-        <v>0.000809423</v>
+        <v>0.002967884333333333</v>
       </c>
       <c r="O3">
-        <v>0.000471795</v>
+        <v>0.001729915</v>
       </c>
       <c r="P3">
-        <v>0.000276629</v>
+        <v>0.001014306333333333</v>
       </c>
       <c r="Q3">
-        <v>0.000162523</v>
+        <v>0.0005959176666666667</v>
       </c>
       <c r="R3">
-        <v>9.37606E-05</v>
+        <v>0.0003437888666666666</v>
       </c>
       <c r="S3">
-        <v>6.09652E-05</v>
+        <v>0.0002235390666666667</v>
       </c>
       <c r="T3">
-        <v>4.94627E-06</v>
+        <v>1.813632333333333E-05</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -745,34 +745,34 @@
         <v>58</v>
       </c>
       <c r="H4">
-        <v>0.0042289086</v>
+        <v>0.0155059982</v>
       </c>
       <c r="I4">
-        <v>0.010519560264239</v>
+        <v>0.03857172096887633</v>
       </c>
       <c r="J4">
-        <v>0.009918797</v>
+        <v>0.03636892233333333</v>
       </c>
       <c r="K4">
-        <v>0.0017512387</v>
+        <v>0.006421208566666666</v>
       </c>
       <c r="L4">
-        <v>0.0003790759</v>
+        <v>0.001389944966666667</v>
       </c>
       <c r="M4">
-        <v>0.00010041517</v>
+        <v>0.0003681889566666667</v>
       </c>
       <c r="N4">
-        <v>2.895889E-05</v>
+        <v>0.0001061825966666667</v>
       </c>
       <c r="O4">
-        <v>9.710926999999999E-06</v>
+        <v>3.560673233333333E-05</v>
       </c>
       <c r="P4">
-        <v>3.47338E-06</v>
+        <v>1.273572666666667E-05</v>
       </c>
       <c r="Q4">
-        <v>3.638875E-09</v>
+        <v>1.334254166666667E-08</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -792,34 +792,34 @@
         <v>58</v>
       </c>
       <c r="H5">
-        <v>0.000136931</v>
+        <v>0.0005020803333333333</v>
       </c>
       <c r="I5">
-        <v>0.00122993</v>
+        <v>0.004509743333333333</v>
       </c>
       <c r="J5">
-        <v>0.00532146</v>
+        <v>0.01951202</v>
       </c>
       <c r="K5">
-        <v>0.00133417</v>
+        <v>0.004891956666666667</v>
       </c>
       <c r="L5">
-        <v>0.00040786</v>
+        <v>0.001495486666666667</v>
       </c>
       <c r="M5">
-        <v>0.000149539</v>
+        <v>0.0005483096666666666</v>
       </c>
       <c r="N5">
-        <v>5.98905E-05</v>
+        <v>0.0002195985</v>
       </c>
       <c r="O5">
-        <v>2.80347E-05</v>
+        <v>0.0001027939</v>
       </c>
       <c r="P5">
-        <v>1.41414E-05</v>
+        <v>5.18518E-05</v>
       </c>
       <c r="Q5">
-        <v>5.70268E-08</v>
+        <v>2.090982666666667E-07</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -839,37 +839,37 @@
         <v>58</v>
       </c>
       <c r="H6">
-        <v>0.0032654782</v>
+        <v>0.01197342006666667</v>
       </c>
       <c r="I6">
-        <v>0.009332263</v>
+        <v>0.03421829766666667</v>
       </c>
       <c r="J6">
-        <v>0.020271443</v>
+        <v>0.07432862433333333</v>
       </c>
       <c r="K6">
-        <v>0.0057054002</v>
+        <v>0.02091980073333333</v>
       </c>
       <c r="L6">
-        <v>0.0014735541</v>
+        <v>0.0054030317</v>
       </c>
       <c r="M6">
-        <v>0.00041607712</v>
+        <v>0.001525616106666667</v>
       </c>
       <c r="N6">
-        <v>0.00011970259</v>
+        <v>0.0004389094966666667</v>
       </c>
       <c r="O6">
-        <v>3.7398267E-05</v>
+        <v>0.000137126979</v>
       </c>
       <c r="P6">
-        <v>1.1431194E-05</v>
+        <v>4.1914378E-05</v>
       </c>
       <c r="Q6">
-        <v>3.875889E-06</v>
+        <v>1.4211593E-05</v>
       </c>
       <c r="R6">
-        <v>5.43614E-10</v>
+        <v>1.993251333333333E-09</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -889,37 +889,37 @@
         <v>58</v>
       </c>
       <c r="H7">
-        <v>0.000107317</v>
+        <v>0.0003934956666666667</v>
       </c>
       <c r="I7">
-        <v>0.0011372</v>
+        <v>0.004169733333333334</v>
       </c>
       <c r="J7">
-        <v>0.009660200000000001</v>
+        <v>0.03542073333333334</v>
       </c>
       <c r="K7">
-        <v>0.00341321</v>
+        <v>0.01251510333333333</v>
       </c>
       <c r="L7">
-        <v>0.0011765</v>
+        <v>0.004313833333333334</v>
       </c>
       <c r="M7">
-        <v>0.000432323</v>
+        <v>0.001585184333333333</v>
       </c>
       <c r="N7">
-        <v>0.000164075</v>
+        <v>0.0006016083333333333</v>
       </c>
       <c r="O7">
-        <v>6.998680000000001E-05</v>
+        <v>0.0002566182666666667</v>
       </c>
       <c r="P7">
-        <v>3.02679E-05</v>
+        <v>0.0001109823</v>
       </c>
       <c r="Q7">
-        <v>1.37367E-05</v>
+        <v>5.03679E-05</v>
       </c>
       <c r="R7">
-        <v>1.02739E-08</v>
+        <v>3.767096666666666E-08</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -939,37 +939,37 @@
         <v>58</v>
       </c>
       <c r="H8">
-        <v>0.011481498</v>
+        <v>0.042098826</v>
       </c>
       <c r="I8">
-        <v>0.0364506125</v>
+        <v>0.1336522458333333</v>
       </c>
       <c r="J8">
-        <v>0.0834476112727499</v>
+        <v>0.3059745746667496</v>
       </c>
       <c r="K8">
-        <v>0.038857160176525</v>
+        <v>0.1424762539805917</v>
       </c>
       <c r="L8">
-        <v>0.012649899</v>
+        <v>0.046382963</v>
       </c>
       <c r="M8">
-        <v>0.004084766</v>
+        <v>0.01497747533333333</v>
       </c>
       <c r="N8">
-        <v>0.0012131931</v>
+        <v>0.0044483747</v>
       </c>
       <c r="O8">
-        <v>0.0003624441</v>
+        <v>0.0013289617</v>
       </c>
       <c r="P8">
-        <v>9.895100000000001E-05</v>
+        <v>0.0003628203333333334</v>
       </c>
       <c r="Q8">
-        <v>2.85771E-05</v>
+        <v>0.0001047827</v>
       </c>
       <c r="R8">
-        <v>8.271133999999999E-06</v>
+        <v>3.032749133333333E-05</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -989,37 +989,37 @@
         <v>58</v>
       </c>
       <c r="H9">
-        <v>0.000435387</v>
+        <v>0.001596419</v>
       </c>
       <c r="I9">
-        <v>0.00480622</v>
+        <v>0.01762280666666667</v>
       </c>
       <c r="J9">
-        <v>0.04103140137779</v>
+        <v>0.1504484717185633</v>
       </c>
       <c r="K9">
-        <v>0.0228907951823</v>
+        <v>0.08393291566843335</v>
       </c>
       <c r="L9">
-        <v>0.00956883</v>
+        <v>0.03508571</v>
       </c>
       <c r="M9">
-        <v>0.00398742</v>
+        <v>0.01462054</v>
       </c>
       <c r="N9">
-        <v>0.00157286</v>
+        <v>0.005767153333333333</v>
       </c>
       <c r="O9">
-        <v>0.000646391</v>
+        <v>0.002370100333333333</v>
       </c>
       <c r="P9">
-        <v>0.000252951</v>
+        <v>0.000927487</v>
       </c>
       <c r="Q9">
-        <v>0.000100102</v>
+        <v>0.0003670406666666667</v>
       </c>
       <c r="R9">
-        <v>3.94679E-05</v>
+        <v>0.0001447156333333334</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1039,49 +1039,49 @@
         <v>58</v>
       </c>
       <c r="F10">
-        <v>0.0001763707</v>
+        <v>0.0006466925666666666</v>
       </c>
       <c r="G10">
-        <v>0.000776877</v>
+        <v>0.002848549</v>
       </c>
       <c r="H10">
-        <v>0.181461231</v>
+        <v>0.665357847</v>
       </c>
       <c r="I10">
-        <v>0.6201593468200001</v>
+        <v>2.273917605006667</v>
       </c>
       <c r="J10">
-        <v>1.3693876490366</v>
+        <v>5.021088046467534</v>
       </c>
       <c r="K10">
-        <v>2.075007090621368</v>
+        <v>7.60835933227835</v>
       </c>
       <c r="L10">
-        <v>2.834564872092171</v>
+        <v>10.39340453100463</v>
       </c>
       <c r="M10">
-        <v>3.71434401577378</v>
+        <v>13.61926139117053</v>
       </c>
       <c r="N10">
-        <v>4.951133202192026</v>
+        <v>18.1541550747041</v>
       </c>
       <c r="O10">
-        <v>6.418000763290171</v>
+        <v>23.53266946539729</v>
       </c>
       <c r="P10">
-        <v>8.151314177805689</v>
+        <v>29.88815198528753</v>
       </c>
       <c r="Q10">
-        <v>10.2577411185936</v>
+        <v>37.6117174348432</v>
       </c>
       <c r="R10">
-        <v>13.34763653572168</v>
+        <v>48.94133396431283</v>
       </c>
       <c r="S10">
-        <v>16.5102337375575</v>
+        <v>60.5375237043775</v>
       </c>
       <c r="T10">
-        <v>19.1065158872959</v>
+        <v>70.05722492008496</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1101,49 +1101,49 @@
         <v>58</v>
       </c>
       <c r="F11">
-        <v>1.12801E-06</v>
+        <v>4.136036666666666E-06</v>
       </c>
       <c r="G11">
-        <v>1.42225E-05</v>
+        <v>5.214916666666667E-05</v>
       </c>
       <c r="H11">
-        <v>0.00734348</v>
+        <v>0.02692609333333333</v>
       </c>
       <c r="I11">
-        <v>0.06659215321</v>
+        <v>0.2441712284366667</v>
       </c>
       <c r="J11">
-        <v>0.5880019046181301</v>
+        <v>2.15600698359981</v>
       </c>
       <c r="K11">
-        <v>1.05897230218907</v>
+        <v>3.882898441359924</v>
       </c>
       <c r="L11">
-        <v>1.58362570839676</v>
+        <v>5.806627597454786</v>
       </c>
       <c r="M11">
-        <v>2.257807589297</v>
+        <v>8.278627827422333</v>
       </c>
       <c r="N11">
-        <v>3.22471778</v>
+        <v>11.82396519333333</v>
       </c>
       <c r="O11">
-        <v>4.789116168939</v>
+        <v>17.560092619443</v>
       </c>
       <c r="P11">
-        <v>7.12236074797</v>
+        <v>26.11532274255667</v>
       </c>
       <c r="Q11">
-        <v>10.6665034525886</v>
+        <v>39.11051265949153</v>
       </c>
       <c r="R11">
-        <v>15.70972829685</v>
+        <v>57.60233708845001</v>
       </c>
       <c r="S11">
-        <v>22.532102579</v>
+        <v>82.61770945633333</v>
       </c>
       <c r="T11">
-        <v>30.37587063</v>
+        <v>111.37819231</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1163,49 +1163,49 @@
         <v>58</v>
       </c>
       <c r="F12">
-        <v>0.00023503322</v>
+        <v>0.0008617884733333334</v>
       </c>
       <c r="G12">
-        <v>0.0011498116</v>
+        <v>0.004215975866666667</v>
       </c>
       <c r="H12">
-        <v>0.138466299</v>
+        <v>0.507709763</v>
       </c>
       <c r="I12">
-        <v>0.5895350133046</v>
+        <v>2.161628382116866</v>
       </c>
       <c r="J12">
-        <v>1.839303340003078</v>
+        <v>6.744112246677953</v>
       </c>
       <c r="K12">
-        <v>2.924851718353088</v>
+        <v>10.72445630062799</v>
       </c>
       <c r="L12">
-        <v>4.168443726545915</v>
+        <v>15.28429366400169</v>
       </c>
       <c r="M12">
-        <v>5.70989031642509</v>
+        <v>20.93626449355866</v>
       </c>
       <c r="N12">
-        <v>7.590291280925047</v>
+        <v>27.83106803005851</v>
       </c>
       <c r="O12">
-        <v>10.16125464065942</v>
+        <v>37.25793368241787</v>
       </c>
       <c r="P12">
-        <v>13.47672817052109</v>
+        <v>49.41466995857734</v>
       </c>
       <c r="Q12">
-        <v>17.7502774716488</v>
+        <v>65.08435072937894</v>
       </c>
       <c r="R12">
-        <v>23.72221199311769</v>
+        <v>86.98144397476486</v>
       </c>
       <c r="S12">
-        <v>30.13320451794228</v>
+        <v>110.4884165657884</v>
       </c>
       <c r="T12">
-        <v>36.108333528775</v>
+        <v>132.3972229388417</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1225,49 +1225,49 @@
         <v>58</v>
       </c>
       <c r="F13">
-        <v>1.46026E-06</v>
+        <v>5.354286666666666E-06</v>
       </c>
       <c r="G13">
-        <v>2.20126E-05</v>
+        <v>8.071286666666666E-05</v>
       </c>
       <c r="H13">
-        <v>0.0063741</v>
+        <v>0.0233717</v>
       </c>
       <c r="I13">
-        <v>0.0666282168653</v>
+        <v>0.2443034618394333</v>
       </c>
       <c r="J13">
-        <v>0.72260110461353</v>
+        <v>2.649537383582943</v>
       </c>
       <c r="K13">
-        <v>1.31371450255099</v>
+        <v>4.816953176020297</v>
       </c>
       <c r="L13">
-        <v>1.96602450905866</v>
+        <v>7.208756533215087</v>
       </c>
       <c r="M13">
-        <v>2.801760428769</v>
+        <v>10.273121572153</v>
       </c>
       <c r="N13">
-        <v>3.97925503</v>
+        <v>14.59060177666667</v>
       </c>
       <c r="O13">
-        <v>5.7745760597292</v>
+        <v>21.1734455523404</v>
       </c>
       <c r="P13">
-        <v>8.408292651869999</v>
+        <v>30.83040639019</v>
       </c>
       <c r="Q13">
-        <v>12.2638532839573</v>
+        <v>44.96746204117677</v>
       </c>
       <c r="R13">
-        <v>17.70835787732</v>
+        <v>64.93064555017334</v>
       </c>
       <c r="S13">
-        <v>25.102517906</v>
+        <v>92.04256565533335</v>
       </c>
       <c r="T13">
-        <v>33.67523282</v>
+        <v>123.4758536733333</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1287,49 +1287,49 @@
         <v>58</v>
       </c>
       <c r="F14">
-        <v>0.00031028649</v>
+        <v>0.00113771713</v>
       </c>
       <c r="G14">
-        <v>0.0013980515</v>
+        <v>0.005126188833333333</v>
       </c>
       <c r="H14">
-        <v>0.31908008062</v>
+        <v>1.169960295606667</v>
       </c>
       <c r="I14">
-        <v>1.266829937171576</v>
+        <v>4.645043102962445</v>
       </c>
       <c r="J14">
-        <v>3.406859272157384</v>
+        <v>12.49181733124374</v>
       </c>
       <c r="K14">
-        <v>4.372814879771613</v>
+        <v>16.03365455916258</v>
       </c>
       <c r="L14">
-        <v>6.332521040407828</v>
+        <v>23.2192438148287</v>
       </c>
       <c r="M14">
-        <v>9.500307936950149</v>
+        <v>34.83446243548388</v>
       </c>
       <c r="N14">
-        <v>12.3744982303509</v>
+        <v>45.37316017795331</v>
       </c>
       <c r="O14">
-        <v>16.49280176782811</v>
+        <v>60.47360648203639</v>
       </c>
       <c r="P14">
-        <v>21.36765173806637</v>
+        <v>78.34805637291002</v>
       </c>
       <c r="Q14">
-        <v>27.7010953659439</v>
+        <v>101.570683008461</v>
       </c>
       <c r="R14">
-        <v>36.90180436162899</v>
+        <v>135.3066159926396</v>
       </c>
       <c r="S14">
-        <v>46.62506273455247</v>
+        <v>170.9585633600257</v>
       </c>
       <c r="T14">
-        <v>55.1941743799258</v>
+        <v>202.3786393930613</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1349,49 +1349,49 @@
         <v>58</v>
       </c>
       <c r="F15">
-        <v>1.8556E-06</v>
+        <v>6.803866666666667E-06</v>
       </c>
       <c r="G15">
-        <v>2.82766E-05</v>
+        <v>0.0001036808666666667</v>
       </c>
       <c r="H15">
-        <v>0.0191935</v>
+        <v>0.07037616666666667</v>
       </c>
       <c r="I15">
-        <v>0.18371458972</v>
+        <v>0.6736201623066665</v>
       </c>
       <c r="J15">
-        <v>1.8609550203128</v>
+        <v>6.823501741146933</v>
       </c>
       <c r="K15">
-        <v>3.2763480041522</v>
+        <v>12.01327601522473</v>
       </c>
       <c r="L15">
-        <v>4.800643010444301</v>
+        <v>17.60235770496243</v>
       </c>
       <c r="M15">
-        <v>6.730275264409</v>
+        <v>24.67767596949967</v>
       </c>
       <c r="N15">
-        <v>9.41101409</v>
+        <v>34.50705166333334</v>
       </c>
       <c r="O15">
-        <v>13.66063751480761</v>
+        <v>50.08900422096124</v>
       </c>
       <c r="P15">
-        <v>20.088403603</v>
+        <v>73.65747987766666</v>
       </c>
       <c r="Q15">
-        <v>29.5997848065207</v>
+        <v>108.5325442905759</v>
       </c>
       <c r="R15">
-        <v>42.63393227362</v>
+        <v>156.3244183366067</v>
       </c>
       <c r="S15">
-        <v>60.40952358</v>
+        <v>221.50158646</v>
       </c>
       <c r="T15">
-        <v>80.30055609999999</v>
+        <v>294.4353723666666</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1411,49 +1411,49 @@
         <v>58</v>
       </c>
       <c r="F16">
-        <v>2.6067401E-05</v>
+        <v>9.558047033333333E-05</v>
       </c>
       <c r="G16">
-        <v>0.00013502965</v>
+        <v>0.0004951087166666667</v>
       </c>
       <c r="H16">
-        <v>0.020798809878065</v>
+        <v>0.07626230288623834</v>
       </c>
       <c r="I16">
-        <v>0.0445891918758</v>
+        <v>0.1634937035446</v>
       </c>
       <c r="J16">
-        <v>0.097351747511516</v>
+        <v>0.3569564075422254</v>
       </c>
       <c r="K16">
-        <v>0.06579974059626201</v>
+        <v>0.2412657155196274</v>
       </c>
       <c r="L16">
-        <v>0.05286807308299001</v>
+        <v>0.1938496013042967</v>
       </c>
       <c r="M16">
-        <v>0.0434315411557909</v>
+        <v>0.1592489842379</v>
       </c>
       <c r="N16">
-        <v>0.033642800120551</v>
+        <v>0.1233569337753537</v>
       </c>
       <c r="O16">
-        <v>0.02724426</v>
+        <v>0.09989561999999999</v>
       </c>
       <c r="P16">
-        <v>0.02032626</v>
+        <v>0.07452961999999999</v>
       </c>
       <c r="Q16">
-        <v>0.01664218</v>
+        <v>0.06102132666666666</v>
       </c>
       <c r="R16">
-        <v>0.01293923</v>
+        <v>0.04744384333333333</v>
       </c>
       <c r="S16">
-        <v>0.01160555</v>
+        <v>0.04255368333333334</v>
       </c>
       <c r="T16">
-        <v>0.008227089999999999</v>
+        <v>0.03016599666666667</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1473,49 +1473,49 @@
         <v>58</v>
       </c>
       <c r="F17">
-        <v>1.99368E-07</v>
+        <v>7.31016E-07</v>
       </c>
       <c r="G17">
-        <v>2.80541E-06</v>
+        <v>1.028650333333333E-05</v>
       </c>
       <c r="H17">
-        <v>0.000979681</v>
+        <v>0.003592163666666667</v>
       </c>
       <c r="I17">
-        <v>0.010173700134741</v>
+        <v>0.037303567160717</v>
       </c>
       <c r="J17">
-        <v>0.09612723916</v>
+        <v>0.3524665435866667</v>
       </c>
       <c r="K17">
-        <v>0.173820268728</v>
+        <v>0.637340985336</v>
       </c>
       <c r="L17">
-        <v>0.2448121309644</v>
+        <v>0.8976444802028</v>
       </c>
       <c r="M17">
-        <v>0.3090072190133</v>
+        <v>1.133026469715434</v>
       </c>
       <c r="N17">
-        <v>0.3644977144337</v>
+        <v>1.336491619590233</v>
       </c>
       <c r="O17">
-        <v>0.4165162391853</v>
+        <v>1.5272262103461</v>
       </c>
       <c r="P17">
-        <v>0.4606675488765</v>
+        <v>1.6891143458805</v>
       </c>
       <c r="Q17">
-        <v>0.5003059399350001</v>
+        <v>1.834455113095</v>
       </c>
       <c r="R17">
-        <v>0.5302695746468999</v>
+        <v>1.9443217737053</v>
       </c>
       <c r="S17">
-        <v>0.559979451925</v>
+        <v>2.053257990391666</v>
       </c>
       <c r="T17">
-        <v>0.5736768135453</v>
+        <v>2.1034816496661</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -1535,49 +1535,49 @@
         <v>58</v>
       </c>
       <c r="F18">
-        <v>2.19499146E-05</v>
+        <v>8.048302020000001E-05</v>
       </c>
       <c r="G18">
-        <v>9.2030148E-05</v>
+        <v>0.000337443876</v>
       </c>
       <c r="H18">
-        <v>0.014274423</v>
+        <v>0.052339551</v>
       </c>
       <c r="I18">
-        <v>0.05192852</v>
+        <v>0.1904045733333333</v>
       </c>
       <c r="J18">
-        <v>0.14414863886957</v>
+        <v>0.5285450091884233</v>
       </c>
       <c r="K18">
-        <v>0.107329680138702</v>
+        <v>0.393542160508574</v>
       </c>
       <c r="L18">
-        <v>0.09795132425766399</v>
+        <v>0.3591548556114346</v>
       </c>
       <c r="M18">
-        <v>0.101619308423745</v>
+        <v>0.372604130887065</v>
       </c>
       <c r="N18">
-        <v>0.0967748084878999</v>
+        <v>0.354840964455633</v>
       </c>
       <c r="O18">
-        <v>0.083206395949395</v>
+        <v>0.305090118481115</v>
       </c>
       <c r="P18">
-        <v>0.06534876809178701</v>
+        <v>0.2396121496698857</v>
       </c>
       <c r="Q18">
-        <v>0.051162416742972</v>
+        <v>0.187595528057564</v>
       </c>
       <c r="R18">
-        <v>0.036425220903268</v>
+        <v>0.1335591433119827</v>
       </c>
       <c r="S18">
-        <v>0.02786968</v>
+        <v>0.1021888266666667</v>
       </c>
       <c r="T18">
-        <v>0.01688567</v>
+        <v>0.06191412333333332</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1597,49 +1597,49 @@
         <v>58</v>
       </c>
       <c r="F19">
-        <v>5.29846E-08</v>
+        <v>1.942768666666667E-07</v>
       </c>
       <c r="G19">
-        <v>6.78073E-07</v>
+        <v>2.486267666666667E-06</v>
       </c>
       <c r="H19">
-        <v>0.000462134</v>
+        <v>0.001694491333333333</v>
       </c>
       <c r="I19">
-        <v>0.00590967</v>
+        <v>0.02166879</v>
       </c>
       <c r="J19">
-        <v>0.0590008002797549</v>
+        <v>0.2163362676924346</v>
       </c>
       <c r="K19">
-        <v>0.0487070027</v>
+        <v>0.1785923432333333</v>
       </c>
       <c r="L19">
-        <v>0.049588862</v>
+        <v>0.1818258273333333</v>
       </c>
       <c r="M19">
-        <v>0.198062800109819</v>
+        <v>0.7262302670693362</v>
       </c>
       <c r="N19">
-        <v>0.248762000190963</v>
+        <v>0.912127334033531</v>
       </c>
       <c r="O19">
-        <v>0.295499500211056</v>
+        <v>1.083498167440539</v>
       </c>
       <c r="P19">
-        <v>0.333081900103577</v>
+        <v>1.221300300379782</v>
       </c>
       <c r="Q19">
-        <v>0.3619562</v>
+        <v>1.327172733333333</v>
       </c>
       <c r="R19">
-        <v>0.3779555</v>
+        <v>1.385836833333333</v>
       </c>
       <c r="S19">
-        <v>0.069828947</v>
+        <v>0.2560394723333334</v>
       </c>
       <c r="T19">
-        <v>0.0430373719441</v>
+        <v>0.1578036971283666</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1659,49 +1659,49 @@
         <v>58</v>
       </c>
       <c r="F20">
-        <v>0.000222441512</v>
+        <v>0.0008156188773333333</v>
       </c>
       <c r="G20">
-        <v>0.00115714258</v>
+        <v>0.004242856126666667</v>
       </c>
       <c r="H20">
-        <v>0.124977350982</v>
+        <v>0.4582502869340001</v>
       </c>
       <c r="I20">
-        <v>0.3215360024447899</v>
+        <v>1.178965342297563</v>
       </c>
       <c r="J20">
-        <v>1.326101432940822</v>
+        <v>4.862371920783014</v>
       </c>
       <c r="K20">
-        <v>1.881102443428024</v>
+        <v>6.897375625902755</v>
       </c>
       <c r="L20">
-        <v>2.755823359871477</v>
+        <v>10.10468565286208</v>
       </c>
       <c r="M20">
-        <v>3.879670977037894</v>
+        <v>14.22546024913894</v>
       </c>
       <c r="N20">
-        <v>5.044604029024</v>
+        <v>18.49688143975467</v>
       </c>
       <c r="O20">
-        <v>6.567026894745263</v>
+        <v>24.07909861406596</v>
       </c>
       <c r="P20">
-        <v>8.277179558714788</v>
+        <v>30.34965838195422</v>
       </c>
       <c r="Q20">
-        <v>10.22377969786102</v>
+        <v>37.48719222549038</v>
       </c>
       <c r="R20">
-        <v>12.26841542851333</v>
+        <v>44.98418990454888</v>
       </c>
       <c r="S20">
-        <v>14.30086906803974</v>
+        <v>52.4365199161457</v>
       </c>
       <c r="T20">
-        <v>15.83870518099903</v>
+        <v>58.07525233032977</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -1721,49 +1721,49 @@
         <v>58</v>
       </c>
       <c r="F21">
-        <v>7.34343E-07</v>
+        <v>2.692591E-06</v>
       </c>
       <c r="G21">
-        <v>1.18368E-05</v>
+        <v>4.34016E-05</v>
       </c>
       <c r="H21">
-        <v>0.00382116</v>
+        <v>0.01401092</v>
       </c>
       <c r="I21">
-        <v>0.0386573</v>
+        <v>0.1417434333333333</v>
       </c>
       <c r="J21">
-        <v>0.467250576217</v>
+        <v>1.713252112795667</v>
       </c>
       <c r="K21">
-        <v>0.898743315509</v>
+        <v>3.295392156866333</v>
       </c>
       <c r="L21">
-        <v>1.37455371843</v>
+        <v>5.04003030091</v>
       </c>
       <c r="M21">
-        <v>1.969551600317857</v>
+        <v>7.221689201165476</v>
       </c>
       <c r="N21">
-        <v>2.8002273162497</v>
+        <v>10.26750015958223</v>
       </c>
       <c r="O21">
-        <v>4.07156465</v>
+        <v>14.92907038333333</v>
       </c>
       <c r="P21">
-        <v>5.85545278</v>
+        <v>21.46999352666667</v>
       </c>
       <c r="Q21">
-        <v>8.341860904955</v>
+        <v>30.58682331816833</v>
       </c>
       <c r="R21">
-        <v>11.730127443169</v>
+        <v>43.01046729161967</v>
       </c>
       <c r="S21">
-        <v>16.196260984</v>
+        <v>59.38629027466666</v>
       </c>
       <c r="T21">
-        <v>21.23404463</v>
+        <v>77.85816364333333</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -1783,43 +1783,43 @@
         <v>58</v>
       </c>
       <c r="H22">
-        <v>0.25997021</v>
+        <v>0.9532241033333332</v>
       </c>
       <c r="I22">
-        <v>1.17897643098</v>
+        <v>4.32291358026</v>
       </c>
       <c r="J22">
-        <v>3.797938543953</v>
+        <v>13.925774661161</v>
       </c>
       <c r="K22">
-        <v>3.1220850609308</v>
+        <v>11.44764522341293</v>
       </c>
       <c r="L22">
-        <v>3.1262937099051</v>
+        <v>11.4630769363187</v>
       </c>
       <c r="M22">
-        <v>12.8103253968109</v>
+        <v>46.97119312163996</v>
       </c>
       <c r="N22">
-        <v>16.55393715836</v>
+        <v>60.69776958065334</v>
       </c>
       <c r="O22">
-        <v>20.281215030849</v>
+        <v>74.364455113113</v>
       </c>
       <c r="P22">
-        <v>23.979208301091</v>
+        <v>87.92376377066698</v>
       </c>
       <c r="Q22">
-        <v>28.30899788117865</v>
+        <v>103.799658897655</v>
       </c>
       <c r="R22">
-        <v>31.1237537429977</v>
+        <v>114.1204303909916</v>
       </c>
       <c r="S22">
-        <v>34.14921683623106</v>
+        <v>125.2137950661805</v>
       </c>
       <c r="T22">
-        <v>35.71165031427138</v>
+        <v>130.942717818995</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -1839,43 +1839,43 @@
         <v>58</v>
       </c>
       <c r="H23">
-        <v>0.0114381</v>
+        <v>0.0419397</v>
       </c>
       <c r="I23">
-        <v>0.148808</v>
+        <v>0.5456293333333333</v>
       </c>
       <c r="J23">
-        <v>1.7044900380059</v>
+        <v>6.249796806021634</v>
       </c>
       <c r="K23">
-        <v>3.11583000923612</v>
+        <v>11.42471003386577</v>
       </c>
       <c r="L23">
-        <v>4.552020015207</v>
+        <v>16.690740055759</v>
       </c>
       <c r="M23">
-        <v>6.2056100945219</v>
+        <v>22.75390367991363</v>
       </c>
       <c r="N23">
-        <v>8.445326764212963</v>
+        <v>30.96619813544753</v>
       </c>
       <c r="O23">
-        <v>11.15390000086555</v>
+        <v>40.89763333650702</v>
       </c>
       <c r="P23">
-        <v>14.15449600382516</v>
+        <v>51.89981868069226</v>
       </c>
       <c r="Q23">
-        <v>17.6292954309917</v>
+        <v>64.64074991363624</v>
       </c>
       <c r="R23">
-        <v>21.470327516476</v>
+        <v>78.72453422707868</v>
       </c>
       <c r="S23">
-        <v>26.072938317</v>
+        <v>95.60077382899999</v>
       </c>
       <c r="T23">
-        <v>30.6346161</v>
+        <v>112.3269257</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -1895,49 +1895,49 @@
         <v>58</v>
       </c>
       <c r="F24">
-        <v>6.534996E-05</v>
+        <v>0.00023961652</v>
       </c>
       <c r="G24">
-        <v>0.00027765754</v>
+        <v>0.001018077646666667</v>
       </c>
       <c r="H24">
-        <v>0.0593651504</v>
+        <v>0.2176722181333333</v>
       </c>
       <c r="I24">
-        <v>0.191132271550778</v>
+        <v>0.7008183290195192</v>
       </c>
       <c r="J24">
-        <v>0.53518891323619</v>
+        <v>1.962359348532696</v>
       </c>
       <c r="K24">
-        <v>0.8409636750068621</v>
+        <v>3.083533475025161</v>
       </c>
       <c r="L24">
-        <v>1.15044662666588</v>
+        <v>4.218304297774893</v>
       </c>
       <c r="M24">
-        <v>1.508840820946296</v>
+        <v>5.532416343469753</v>
       </c>
       <c r="N24">
-        <v>2.007773654817256</v>
+        <v>7.361836734329939</v>
       </c>
       <c r="O24">
-        <v>2.644412044349891</v>
+        <v>9.6961774959496</v>
       </c>
       <c r="P24">
-        <v>3.452248204997141</v>
+        <v>12.65824341832285</v>
       </c>
       <c r="Q24">
-        <v>4.51627906000037</v>
+        <v>16.55968988666802</v>
       </c>
       <c r="R24">
-        <v>6.005408625617015</v>
+        <v>22.01983162726239</v>
       </c>
       <c r="S24">
-        <v>7.593414820344879</v>
+        <v>27.84252100793123</v>
       </c>
       <c r="T24">
-        <v>8.847325374455</v>
+        <v>32.44019303966833</v>
       </c>
     </row>
     <row r="25" spans="1:20">
@@ -1957,49 +1957,49 @@
         <v>58</v>
       </c>
       <c r="F25">
-        <v>3.94189E-07</v>
+        <v>1.445359666666667E-06</v>
       </c>
       <c r="G25">
-        <v>5.17251E-06</v>
+        <v>1.896587E-05</v>
       </c>
       <c r="H25">
-        <v>0.00299682</v>
+        <v>0.01098834</v>
       </c>
       <c r="I25">
-        <v>0.0220742145229</v>
+        <v>0.08093878658396667</v>
       </c>
       <c r="J25">
-        <v>0.23812190236471</v>
+        <v>0.8731136420039367</v>
       </c>
       <c r="K25">
-        <v>0.416372100582724</v>
+        <v>1.526697702136655</v>
       </c>
       <c r="L25">
-        <v>0.62187440165938</v>
+        <v>2.280206139417727</v>
       </c>
       <c r="M25">
-        <v>0.871877032436</v>
+        <v>3.196882452265333</v>
       </c>
       <c r="N25">
-        <v>1.218169026</v>
+        <v>4.466619762</v>
       </c>
       <c r="O25">
-        <v>1.76602584108064</v>
+        <v>6.475428083962346</v>
       </c>
       <c r="P25">
-        <v>2.554109124309</v>
+        <v>9.365066789133</v>
       </c>
       <c r="Q25">
-        <v>3.71071004495747</v>
+        <v>13.60593683151072</v>
       </c>
       <c r="R25">
-        <v>5.26228990137</v>
+        <v>19.29506297169</v>
       </c>
       <c r="S25">
-        <v>7.286839043</v>
+        <v>26.71840982433333</v>
       </c>
       <c r="T25">
-        <v>9.22679323</v>
+        <v>33.83157517666667</v>
       </c>
     </row>
     <row r="26" spans="1:20">
@@ -2019,49 +2019,49 @@
         <v>58</v>
       </c>
       <c r="F26">
-        <v>5.2394201E-06</v>
+        <v>1.921120703333333E-05</v>
       </c>
       <c r="G26">
-        <v>2.2209544E-05</v>
+        <v>8.143499466666667E-05</v>
       </c>
       <c r="H26">
-        <v>0.0024480439</v>
+        <v>0.008976160966666666</v>
       </c>
       <c r="I26">
-        <v>0.0058156748</v>
+        <v>0.02132414093333333</v>
       </c>
       <c r="J26">
-        <v>0.005139057099999999</v>
+        <v>0.01884320936666667</v>
       </c>
       <c r="K26">
-        <v>0.00124757</v>
+        <v>0.004574423333333333</v>
       </c>
       <c r="L26">
-        <v>0.00043023069</v>
+        <v>0.00157751253</v>
       </c>
       <c r="M26">
-        <v>0.00019846444</v>
+        <v>0.0007277029466666666</v>
       </c>
       <c r="N26">
-        <v>0.00011402226</v>
+        <v>0.00041808162</v>
       </c>
       <c r="O26">
-        <v>7.840846999999999E-05</v>
+        <v>0.0002874977233333333</v>
       </c>
       <c r="P26">
-        <v>5.65571E-05</v>
+        <v>0.0002073760333333334</v>
       </c>
       <c r="Q26">
-        <v>4.36375E-05</v>
+        <v>0.0001600041666666667</v>
       </c>
       <c r="R26">
-        <v>3.467828E-05</v>
+        <v>0.0001271536933333333</v>
       </c>
       <c r="S26">
-        <v>3.078231E-05</v>
+        <v>0.00011286847</v>
       </c>
       <c r="T26">
-        <v>2.063451E-05</v>
+        <v>7.565986999999999E-05</v>
       </c>
     </row>
     <row r="27" spans="1:20">
@@ -2081,49 +2081,49 @@
         <v>58</v>
       </c>
       <c r="F27">
-        <v>2.11768E-08</v>
+        <v>7.764826666666667E-08</v>
       </c>
       <c r="G27">
-        <v>2.70462E-07</v>
+        <v>9.91694E-07</v>
       </c>
       <c r="H27">
-        <v>7.22456E-05</v>
+        <v>0.0002649005333333333</v>
       </c>
       <c r="I27">
-        <v>0.000573468</v>
+        <v>0.002102716</v>
       </c>
       <c r="J27">
-        <v>0.00239636</v>
+        <v>0.008786653333333333</v>
       </c>
       <c r="K27">
-        <v>0.000766925</v>
+        <v>0.002812058333333334</v>
       </c>
       <c r="L27">
-        <v>0.000336986</v>
+        <v>0.001235615333333333</v>
       </c>
       <c r="M27">
-        <v>0.000193367</v>
+        <v>0.0007090123333333333</v>
       </c>
       <c r="N27">
-        <v>0.000140758</v>
+        <v>0.0005161126666666666</v>
       </c>
       <c r="O27">
-        <v>0.000119093</v>
+        <v>0.0004366743333333333</v>
       </c>
       <c r="P27">
-        <v>0.000105335</v>
+        <v>0.0003862283333333333</v>
       </c>
       <c r="Q27">
-        <v>9.819250000000001E-05</v>
+        <v>0.0003600391666666667</v>
       </c>
       <c r="R27">
-        <v>9.238659999999999E-05</v>
+        <v>0.0003387508666666667</v>
       </c>
       <c r="S27">
-        <v>9.66834E-05</v>
+        <v>0.0003545058</v>
       </c>
       <c r="T27">
-        <v>8.07161E-05</v>
+        <v>0.0002959590333333333</v>
       </c>
     </row>
     <row r="28" spans="1:20">
@@ -2143,46 +2143,46 @@
         <v>58</v>
       </c>
       <c r="F28">
-        <v>1.2327609E-05</v>
+        <v>4.520123299999999E-05</v>
       </c>
       <c r="G28">
-        <v>5.956538899999999E-05</v>
+        <v>0.0002184064263333333</v>
       </c>
       <c r="H28">
-        <v>0.007486560000000001</v>
+        <v>0.02745072</v>
       </c>
       <c r="I28">
-        <v>0.017459462</v>
+        <v>0.06401802733333332</v>
       </c>
       <c r="J28">
-        <v>0.013489756</v>
+        <v>0.04946243866666666</v>
       </c>
       <c r="K28">
-        <v>0.00282698</v>
+        <v>0.01036559333333333</v>
       </c>
       <c r="L28">
-        <v>0.0008587175</v>
+        <v>0.003148630833333333</v>
       </c>
       <c r="M28">
-        <v>0.0003447173</v>
+        <v>0.001263963433333333</v>
       </c>
       <c r="N28">
-        <v>0.0001657922</v>
+        <v>0.0006079047333333333</v>
       </c>
       <c r="O28">
-        <v>9.565669E-05</v>
+        <v>0.0003507411966666667</v>
       </c>
       <c r="P28">
-        <v>5.914383E-05</v>
+        <v>0.00021686071</v>
       </c>
       <c r="Q28">
-        <v>3.960876E-05</v>
+        <v>0.00014523212</v>
       </c>
       <c r="R28">
-        <v>2.712103E-05</v>
+        <v>9.944377666666667E-05</v>
       </c>
       <c r="S28">
-        <v>7.59122E-07</v>
+        <v>2.783447333333333E-06</v>
       </c>
     </row>
     <row r="29" spans="1:20">
@@ -2202,46 +2202,46 @@
         <v>58</v>
       </c>
       <c r="F29">
-        <v>8.55488E-08</v>
+        <v>3.136789333333333E-07</v>
       </c>
       <c r="G29">
-        <v>1.20271E-06</v>
+        <v>4.409936666666667E-06</v>
       </c>
       <c r="H29">
-        <v>0.000428443</v>
+        <v>0.001570957666666667</v>
       </c>
       <c r="I29">
-        <v>0.00270545</v>
+        <v>0.009919983333333333</v>
       </c>
       <c r="J29">
-        <v>0.009114560000000001</v>
+        <v>0.03342005333333334</v>
       </c>
       <c r="K29">
-        <v>0.00254774</v>
+        <v>0.009341713333333333</v>
       </c>
       <c r="L29">
-        <v>0.0009996149999999999</v>
+        <v>0.003665255</v>
       </c>
       <c r="M29">
-        <v>0.000509652</v>
+        <v>0.001868724</v>
       </c>
       <c r="N29">
-        <v>0.000307818</v>
+        <v>0.001128666</v>
       </c>
       <c r="O29">
-        <v>0.000219513</v>
+        <v>0.000804881</v>
       </c>
       <c r="P29">
-        <v>0.000169599</v>
+        <v>0.000621863</v>
       </c>
       <c r="Q29">
-        <v>0.000138138</v>
+        <v>0.000506506</v>
       </c>
       <c r="R29">
-        <v>0.000112946</v>
+        <v>0.0004141353333333333</v>
       </c>
       <c r="S29">
-        <v>6.35839E-06</v>
+        <v>2.331409666666667E-05</v>
       </c>
     </row>
     <row r="30" spans="1:20">
@@ -2261,34 +2261,34 @@
         <v>58</v>
       </c>
       <c r="H30">
-        <v>0.0024472275</v>
+        <v>0.0089731675</v>
       </c>
       <c r="I30">
-        <v>0.004836131</v>
+        <v>0.01773248033333334</v>
       </c>
       <c r="J30">
-        <v>0.0030377525</v>
+        <v>0.01113842583333333</v>
       </c>
       <c r="K30">
-        <v>0.00051742382</v>
+        <v>0.001897220673333333</v>
       </c>
       <c r="L30">
-        <v>0.00012587521</v>
+        <v>0.0004615424366666666</v>
       </c>
       <c r="M30">
-        <v>4.0466471E-05</v>
+        <v>0.0001483770603333333</v>
       </c>
       <c r="N30">
-        <v>1.6035819E-05</v>
+        <v>5.8798003E-05</v>
       </c>
       <c r="O30">
-        <v>7.702281E-06</v>
+        <v>2.8241697E-05</v>
       </c>
       <c r="P30">
-        <v>3.960885E-06</v>
+        <v>1.4523245E-05</v>
       </c>
       <c r="Q30">
-        <v>4.874111E-07</v>
+        <v>1.787174033333333E-06</v>
       </c>
     </row>
     <row r="31" spans="1:20">
@@ -2308,34 +2308,34 @@
         <v>58</v>
       </c>
       <c r="H31">
-        <v>6.5503E-05</v>
+        <v>0.0002401776666666667</v>
       </c>
       <c r="I31">
-        <v>0.000482176</v>
+        <v>0.001767978666666667</v>
       </c>
       <c r="J31">
-        <v>0.00150935</v>
+        <v>0.005534283333333333</v>
       </c>
       <c r="K31">
-        <v>0.000342501</v>
+        <v>0.001255837</v>
       </c>
       <c r="L31">
-        <v>0.000110605</v>
+        <v>0.0004055516666666667</v>
       </c>
       <c r="M31">
-        <v>4.67686E-05</v>
+        <v>0.0001714848666666667</v>
       </c>
       <c r="N31">
-        <v>2.51559E-05</v>
+        <v>9.22383E-05</v>
       </c>
       <c r="O31">
-        <v>1.59331E-05</v>
+        <v>5.842136666666667E-05</v>
       </c>
       <c r="P31">
-        <v>1.07095E-05</v>
+        <v>3.926816666666666E-05</v>
       </c>
       <c r="Q31">
-        <v>2.11568E-06</v>
+        <v>7.757493333333332E-06</v>
       </c>
     </row>
     <row r="32" spans="1:20">
@@ -2355,49 +2355,49 @@
         <v>58</v>
       </c>
       <c r="F32">
-        <v>2.4667522E-06</v>
+        <v>9.044758066666667E-06</v>
       </c>
       <c r="G32">
-        <v>9.596063999999999E-06</v>
+        <v>3.5185568E-05</v>
       </c>
       <c r="H32">
-        <v>0.0012507884</v>
+        <v>0.004586224133333333</v>
       </c>
       <c r="I32">
-        <v>0.00461628253</v>
+        <v>0.01692636927666667</v>
       </c>
       <c r="J32">
-        <v>0.009069787787740001</v>
+        <v>0.03325588855504667</v>
       </c>
       <c r="K32">
-        <v>0.002996394</v>
+        <v>0.010986778</v>
       </c>
       <c r="L32">
-        <v>0.001160375</v>
+        <v>0.004254708333333333</v>
       </c>
       <c r="M32">
-        <v>0.000565381</v>
+        <v>0.002073063666666667</v>
       </c>
       <c r="N32">
-        <v>0.0003238661</v>
+        <v>0.001187509033333333</v>
       </c>
       <c r="O32">
-        <v>0.0002257995</v>
+        <v>0.0008279315</v>
       </c>
       <c r="P32">
-        <v>0.0001596679</v>
+        <v>0.0005854489666666665</v>
       </c>
       <c r="Q32">
-        <v>0.0001192439</v>
+        <v>0.0004372276333333334</v>
       </c>
       <c r="R32">
-        <v>8.734649999999999E-05</v>
+        <v>0.0003202705</v>
       </c>
       <c r="S32">
-        <v>8.309309999999999E-05</v>
+        <v>0.0003046747</v>
       </c>
       <c r="T32">
-        <v>6.10784E-05</v>
+        <v>0.0002239541333333333</v>
       </c>
     </row>
     <row r="33" spans="1:20">
@@ -2417,49 +2417,49 @@
         <v>58</v>
       </c>
       <c r="F33">
-        <v>3.68326E-08</v>
+        <v>1.350528666666667E-07</v>
       </c>
       <c r="G33">
-        <v>4.23173E-07</v>
+        <v>1.551634333333333E-06</v>
       </c>
       <c r="H33">
-        <v>0.00015234</v>
+        <v>0.00055858</v>
       </c>
       <c r="I33">
-        <v>0.0011408547749</v>
+        <v>0.004183134174633334</v>
       </c>
       <c r="J33">
-        <v>0.0063758382412</v>
+        <v>0.02337807355106667</v>
       </c>
       <c r="K33">
-        <v>0.00265059531702</v>
+        <v>0.009718849495740001</v>
       </c>
       <c r="L33">
-        <v>0.00125706</v>
+        <v>0.00460922</v>
       </c>
       <c r="M33">
-        <v>0.000731768</v>
+        <v>0.002683149333333334</v>
       </c>
       <c r="N33">
-        <v>0.000485997</v>
+        <v>0.001781989</v>
       </c>
       <c r="O33">
-        <v>0.000392737</v>
+        <v>0.001440035666666667</v>
       </c>
       <c r="P33">
-        <v>0.000328431</v>
+        <v>0.001204247</v>
       </c>
       <c r="Q33">
-        <v>0.000292212</v>
+        <v>0.001071444</v>
       </c>
       <c r="R33">
-        <v>0.000250088</v>
+        <v>0.0009169893333333333</v>
       </c>
       <c r="S33">
-        <v>0.000241941</v>
+        <v>0.0008871169999999999</v>
       </c>
       <c r="T33">
-        <v>0.000201227</v>
+        <v>0.0007378323333333334</v>
       </c>
     </row>
     <row r="34" spans="1:20">
@@ -2479,37 +2479,37 @@
         <v>58</v>
       </c>
       <c r="F34">
-        <v>8.1651842E-06</v>
+        <v>2.993900873333334E-05</v>
       </c>
       <c r="G34">
-        <v>2.8300187E-05</v>
+        <v>0.0001037673523333333</v>
       </c>
       <c r="H34">
-        <v>0.0043654681</v>
+        <v>0.01600671636666667</v>
       </c>
       <c r="I34">
-        <v>0.0062343357</v>
+        <v>0.0228592309</v>
       </c>
       <c r="J34">
-        <v>0.0038174102</v>
+        <v>0.01399717073333333</v>
       </c>
       <c r="K34">
-        <v>0.0006607034799999999</v>
+        <v>0.002422579426666667</v>
       </c>
       <c r="L34">
-        <v>0.00017589212</v>
+        <v>0.0006449377733333333</v>
       </c>
       <c r="M34">
-        <v>6.4870737E-05</v>
+        <v>0.000237859369</v>
       </c>
       <c r="N34">
-        <v>2.592532E-05</v>
+        <v>9.505950666666667E-05</v>
       </c>
       <c r="O34">
-        <v>1.2393333E-05</v>
+        <v>4.5442221E-05</v>
       </c>
       <c r="P34">
-        <v>6.449556000000001E-06</v>
+        <v>2.3648372E-05</v>
       </c>
     </row>
     <row r="35" spans="1:20">
@@ -2529,40 +2529,40 @@
         <v>58</v>
       </c>
       <c r="F35">
-        <v>2.82387E-08</v>
+        <v>1.035419E-07</v>
       </c>
       <c r="G35">
-        <v>3.19497E-07</v>
+        <v>1.171489E-06</v>
       </c>
       <c r="H35">
-        <v>9.3552E-05</v>
+        <v>0.000343024</v>
       </c>
       <c r="I35">
-        <v>0.000501661</v>
+        <v>0.001839423666666667</v>
       </c>
       <c r="J35">
-        <v>0.00170667</v>
+        <v>0.00625779</v>
       </c>
       <c r="K35">
-        <v>0.000411759</v>
+        <v>0.001509783</v>
       </c>
       <c r="L35">
-        <v>0.000148491</v>
+        <v>0.000544467</v>
       </c>
       <c r="M35">
-        <v>7.19432E-05</v>
+        <v>0.0002637917333333333</v>
       </c>
       <c r="N35">
-        <v>3.9865E-05</v>
+        <v>0.0001461716666666667</v>
       </c>
       <c r="O35">
-        <v>2.5762E-05</v>
+        <v>9.446066666666667E-05</v>
       </c>
       <c r="P35">
-        <v>1.77935E-05</v>
+        <v>6.524283333333334E-05</v>
       </c>
       <c r="Q35">
-        <v>1.82876E-10</v>
+        <v>6.705453333333335E-10</v>
       </c>
     </row>
     <row r="36" spans="1:20">
@@ -2582,31 +2582,31 @@
         <v>58</v>
       </c>
       <c r="F36">
-        <v>2.74150107E-06</v>
+        <v>1.005217059E-05</v>
       </c>
       <c r="G36">
-        <v>1.01346849E-05</v>
+        <v>3.71605113E-05</v>
       </c>
       <c r="H36">
-        <v>0.00109602048</v>
+        <v>0.004018741760000001</v>
       </c>
       <c r="I36">
-        <v>0.00041015576</v>
+        <v>0.001503904453333333</v>
       </c>
       <c r="J36">
-        <v>0.00014303448</v>
+        <v>0.00052445976</v>
       </c>
       <c r="K36">
-        <v>1.6103207E-05</v>
+        <v>5.904509233333333E-05</v>
       </c>
       <c r="L36">
-        <v>2.9992782E-06</v>
+        <v>1.09973534E-05</v>
       </c>
       <c r="M36">
-        <v>7.870234E-07</v>
+        <v>2.885752466666666E-06</v>
       </c>
       <c r="N36">
-        <v>3.453809E-08</v>
+        <v>1.266396633333333E-07</v>
       </c>
     </row>
     <row r="37" spans="1:20">
@@ -2626,31 +2626,31 @@
         <v>58</v>
       </c>
       <c r="F37">
-        <v>5.99106E-09</v>
+        <v>2.196722E-08</v>
       </c>
       <c r="G37">
-        <v>8.39482E-08</v>
+        <v>3.078100666666667E-07</v>
       </c>
       <c r="H37">
-        <v>2.66652E-05</v>
+        <v>9.77724E-05</v>
       </c>
       <c r="I37">
-        <v>4.31269E-05</v>
+        <v>0.0001581319666666667</v>
       </c>
       <c r="J37">
-        <v>8.7055E-05</v>
+        <v>0.0003192016666666667</v>
       </c>
       <c r="K37">
-        <v>1.45626E-05</v>
+        <v>5.33962E-05</v>
       </c>
       <c r="L37">
-        <v>3.98938E-06</v>
+        <v>1.462772666666667E-05</v>
       </c>
       <c r="M37">
-        <v>1.53334E-06</v>
+        <v>5.622246666666667E-06</v>
       </c>
       <c r="N37">
-        <v>1.42657E-07</v>
+        <v>5.230756666666666E-07</v>
       </c>
     </row>
     <row r="38" spans="1:20">
@@ -2670,49 +2670,49 @@
         <v>58</v>
       </c>
       <c r="F38">
-        <v>1.1379414E-05</v>
+        <v>4.1724518E-05</v>
       </c>
       <c r="G38">
-        <v>6.0861101E-05</v>
+        <v>0.0002231573703333333</v>
       </c>
       <c r="H38">
-        <v>0.010055753</v>
+        <v>0.03687109433333333</v>
       </c>
       <c r="I38">
-        <v>0.02931943938517</v>
+        <v>0.1075046110789567</v>
       </c>
       <c r="J38">
-        <v>0.07156186194351</v>
+        <v>0.26239349379287</v>
       </c>
       <c r="K38">
-        <v>0.027648446</v>
+        <v>0.1013776353333333</v>
       </c>
       <c r="L38">
-        <v>0.012944576</v>
+        <v>0.04746344533333333</v>
       </c>
       <c r="M38">
-        <v>0.007480442</v>
+        <v>0.02742828733333333</v>
       </c>
       <c r="N38">
-        <v>0.005389657</v>
+        <v>0.01976207566666667</v>
       </c>
       <c r="O38">
-        <v>0.004311788</v>
+        <v>0.01580988933333333</v>
       </c>
       <c r="P38">
-        <v>0.003435668</v>
+        <v>0.01259744933333333</v>
       </c>
       <c r="Q38">
-        <v>0.002946436</v>
+        <v>0.01080359866666667</v>
       </c>
       <c r="R38">
-        <v>0.002408891</v>
+        <v>0.008832600333333334</v>
       </c>
       <c r="S38">
-        <v>0.002401383</v>
+        <v>0.008805071000000001</v>
       </c>
       <c r="T38">
-        <v>0.001875613</v>
+        <v>0.006877247666666666</v>
       </c>
     </row>
     <row r="39" spans="1:20">
@@ -2732,49 +2732,49 @@
         <v>58</v>
       </c>
       <c r="F39">
-        <v>7.37246E-08</v>
+        <v>2.703235333333334E-07</v>
       </c>
       <c r="G39">
-        <v>1.19742E-06</v>
+        <v>4.39054E-06</v>
       </c>
       <c r="H39">
-        <v>0.000442509</v>
+        <v>0.001622533</v>
       </c>
       <c r="I39">
-        <v>0.00419626</v>
+        <v>0.01538628666666667</v>
       </c>
       <c r="J39">
-        <v>0.0378336</v>
+        <v>0.1387232</v>
       </c>
       <c r="K39">
-        <v>0.017368900453557</v>
+        <v>0.06368596832970901</v>
       </c>
       <c r="L39">
-        <v>0.00980382</v>
+        <v>0.03594734</v>
       </c>
       <c r="M39">
-        <v>0.00672501</v>
+        <v>0.02465837</v>
       </c>
       <c r="N39">
-        <v>0.00620617</v>
+        <v>0.02275595666666666</v>
       </c>
       <c r="O39">
-        <v>0.00602653</v>
+        <v>0.02209727666666667</v>
       </c>
       <c r="P39">
-        <v>0.00572218</v>
+        <v>0.02098132666666667</v>
       </c>
       <c r="Q39">
-        <v>0.00524749</v>
+        <v>0.01924079666666667</v>
       </c>
       <c r="R39">
-        <v>0.00482067</v>
+        <v>0.01767579</v>
       </c>
       <c r="S39">
-        <v>0.00515278</v>
+        <v>0.01889352666666667</v>
       </c>
       <c r="T39">
-        <v>0.00482896</v>
+        <v>0.01770618666666667</v>
       </c>
     </row>
     <row r="40" spans="1:20">
@@ -2794,49 +2794,49 @@
         <v>58</v>
       </c>
       <c r="F40">
-        <v>0.00012789655</v>
+        <v>0.0004689540166666666</v>
       </c>
       <c r="G40">
-        <v>0.00054157124</v>
+        <v>0.001985761213333334</v>
       </c>
       <c r="H40">
-        <v>0.114296629</v>
+        <v>0.4190876396666667</v>
       </c>
       <c r="I40">
-        <v>0.3810252232946</v>
+        <v>1.397092485413533</v>
       </c>
       <c r="J40">
-        <v>1.20472279824105</v>
+        <v>4.417316926883849</v>
       </c>
       <c r="K40">
-        <v>1.842010121103514</v>
+        <v>6.754037110712884</v>
       </c>
       <c r="L40">
-        <v>2.549101341596859</v>
+        <v>9.346704919188484</v>
       </c>
       <c r="M40">
-        <v>3.35626653386892</v>
+        <v>12.30631062418604</v>
       </c>
       <c r="N40">
-        <v>4.349972877293256</v>
+        <v>15.94990055007527</v>
       </c>
       <c r="O40">
-        <v>5.665244408082994</v>
+        <v>20.77256282963765</v>
       </c>
       <c r="P40">
-        <v>7.234316798262171</v>
+        <v>26.52582826029463</v>
       </c>
       <c r="Q40">
-        <v>9.10141337930785</v>
+        <v>33.37184905746211</v>
       </c>
       <c r="R40">
-        <v>10.8397568383858</v>
+        <v>39.74577507408127</v>
       </c>
       <c r="S40">
-        <v>12.4171453737224</v>
+        <v>45.52953303698214</v>
       </c>
       <c r="T40">
-        <v>13.29062707737596</v>
+        <v>48.73229928371185</v>
       </c>
     </row>
     <row r="41" spans="1:20">
@@ -2856,49 +2856,49 @@
         <v>58</v>
       </c>
       <c r="F41">
-        <v>7.547689999999999E-07</v>
+        <v>2.767486333333333E-06</v>
       </c>
       <c r="G41">
-        <v>9.11825E-06</v>
+        <v>3.343358333333333E-05</v>
       </c>
       <c r="H41">
-        <v>0.00391517</v>
+        <v>0.01435562333333333</v>
       </c>
       <c r="I41">
-        <v>0.0340549042555</v>
+        <v>0.1248679822701667</v>
       </c>
       <c r="J41">
-        <v>0.39966300419517</v>
+        <v>1.46543101538229</v>
       </c>
       <c r="K41">
-        <v>0.72318610174977</v>
+        <v>2.65168237308249</v>
       </c>
       <c r="L41">
-        <v>1.07818590686889</v>
+        <v>3.95334832518593</v>
       </c>
       <c r="M41">
-        <v>1.51712471734</v>
+        <v>5.562790630246667</v>
       </c>
       <c r="N41">
-        <v>2.10968154</v>
+        <v>7.73549898</v>
       </c>
       <c r="O41">
-        <v>3.00077635510119</v>
+        <v>11.00284663537103</v>
       </c>
       <c r="P41">
-        <v>4.23218619299</v>
+        <v>15.51801604096333</v>
       </c>
       <c r="Q41">
-        <v>5.901989134820592</v>
+        <v>21.6406268276755</v>
       </c>
       <c r="R41">
-        <v>7.74398222465</v>
+        <v>28.39460149038333</v>
       </c>
       <c r="S41">
-        <v>9.625562646000001</v>
+        <v>35.293729702</v>
       </c>
       <c r="T41">
-        <v>11.11916953</v>
+        <v>40.77028827666667</v>
       </c>
     </row>
     <row r="42" spans="1:20">
@@ -2918,49 +2918,49 @@
         <v>58</v>
       </c>
       <c r="F42">
-        <v>0.000119607312</v>
+        <v>0.000438560144</v>
       </c>
       <c r="G42">
-        <v>0.00044882435</v>
+        <v>0.001645689283333333</v>
       </c>
       <c r="H42">
-        <v>0.066978614356</v>
+        <v>0.2455882526386667</v>
       </c>
       <c r="I42">
-        <v>0.25352357161137</v>
+        <v>0.92958642924169</v>
       </c>
       <c r="J42">
-        <v>0.698198155200801</v>
+        <v>2.560059902402937</v>
       </c>
       <c r="K42">
-        <v>0.7812183310255001</v>
+        <v>2.864467213760167</v>
       </c>
       <c r="L42">
-        <v>0.48978151604454</v>
+        <v>1.79586555882998</v>
       </c>
       <c r="M42">
-        <v>0.391790148096181</v>
+        <v>1.436563876352664</v>
       </c>
       <c r="N42">
-        <v>0.301591182518845</v>
+        <v>1.105834335902432</v>
       </c>
       <c r="O42">
-        <v>0.244030332905322</v>
+        <v>0.8947778873195139</v>
       </c>
       <c r="P42">
-        <v>0.1840111940859499</v>
+        <v>0.6747077116484829</v>
       </c>
       <c r="Q42">
-        <v>0.1350213926582039</v>
+        <v>0.4950784397467476</v>
       </c>
       <c r="R42">
-        <v>0.09585921</v>
+        <v>0.35148377</v>
       </c>
       <c r="S42">
-        <v>0.07119391999999999</v>
+        <v>0.2610443733333334</v>
       </c>
       <c r="T42">
-        <v>0.04354843</v>
+        <v>0.1596775766666667</v>
       </c>
     </row>
     <row r="43" spans="1:20">
@@ -2980,49 +2980,49 @@
         <v>58</v>
       </c>
       <c r="F43">
-        <v>4.58455E-07</v>
+        <v>1.681001666666667E-06</v>
       </c>
       <c r="G43">
-        <v>5.58151E-06</v>
+        <v>2.046553666666666E-05</v>
       </c>
       <c r="H43">
-        <v>0.00203593</v>
+        <v>0.007465076666666667</v>
       </c>
       <c r="I43">
-        <v>0.0258288</v>
+        <v>0.0947056</v>
       </c>
       <c r="J43">
-        <v>0.2787770124174</v>
+        <v>1.0221823788638</v>
       </c>
       <c r="K43">
-        <v>0.50506800232323</v>
+        <v>1.85191600851851</v>
       </c>
       <c r="L43">
-        <v>0.721771002255</v>
+        <v>2.646493674935</v>
       </c>
       <c r="M43">
-        <v>0.8299510007920871</v>
+        <v>3.043153669570986</v>
       </c>
       <c r="N43">
-        <v>0.210162440349446</v>
+        <v>0.7705956146146353</v>
       </c>
       <c r="O43">
-        <v>0.1988015112013169</v>
+        <v>0.7289388744048285</v>
       </c>
       <c r="P43">
-        <v>0.17725187615</v>
+        <v>0.6499235458833333</v>
       </c>
       <c r="Q43">
-        <v>0.153574172417</v>
+        <v>0.5631052988623333</v>
       </c>
       <c r="R43">
-        <v>0.1279382652597999</v>
+        <v>0.4691069726192663</v>
       </c>
       <c r="S43">
-        <v>0.11326807098802</v>
+        <v>0.4153162602894067</v>
       </c>
       <c r="T43">
-        <v>0.087083408173789</v>
+        <v>0.3193058299705597</v>
       </c>
     </row>
     <row r="44" spans="1:20">
@@ -3042,19 +3042,19 @@
         <v>58</v>
       </c>
       <c r="H44">
-        <v>0.00045428613</v>
+        <v>0.00166571581</v>
       </c>
       <c r="I44">
-        <v>0.00026791012</v>
+        <v>0.0009823371066666668</v>
       </c>
       <c r="J44">
-        <v>4.8115614E-05</v>
+        <v>0.000176423918</v>
       </c>
       <c r="K44">
-        <v>2.2850003E-06</v>
+        <v>8.378334433333333E-06</v>
       </c>
       <c r="L44">
-        <v>1.481989E-07</v>
+        <v>5.433959666666667E-07</v>
       </c>
     </row>
     <row r="45" spans="1:20">
@@ -3074,19 +3074,19 @@
         <v>58</v>
       </c>
       <c r="H45">
-        <v>1.73178E-05</v>
+        <v>6.34986E-05</v>
       </c>
       <c r="I45">
-        <v>4.46258E-05</v>
+        <v>0.0001636279333333333</v>
       </c>
       <c r="J45">
-        <v>5.22055E-05</v>
+        <v>0.0001914201666666667</v>
       </c>
       <c r="K45">
-        <v>4.40278E-06</v>
+        <v>1.614352666666667E-05</v>
       </c>
       <c r="L45">
-        <v>5.12156E-07</v>
+        <v>1.877905333333334E-06</v>
       </c>
     </row>
     <row r="46" spans="1:20">
@@ -3106,43 +3106,43 @@
         <v>58</v>
       </c>
       <c r="H46">
-        <v>0.071877071</v>
+        <v>0.2635492603333333</v>
       </c>
       <c r="I46">
-        <v>0.31786599</v>
+        <v>1.16550863</v>
       </c>
       <c r="J46">
-        <v>0.687604920606</v>
+        <v>2.521218042222</v>
       </c>
       <c r="K46">
-        <v>1.1414333178769</v>
+        <v>4.185255498881967</v>
       </c>
       <c r="L46">
-        <v>0.46672531366603</v>
+        <v>1.711326150108776</v>
       </c>
       <c r="M46">
-        <v>0.41062487585067</v>
+        <v>1.50562454478579</v>
       </c>
       <c r="N46">
-        <v>0.346958900495601</v>
+        <v>1.272182635150537</v>
       </c>
       <c r="O46">
-        <v>0.313813741145772</v>
+        <v>1.150650384201164</v>
       </c>
       <c r="P46">
-        <v>0.26326964539274</v>
+        <v>0.9653220331067133</v>
       </c>
       <c r="Q46">
-        <v>0.214461368736779</v>
+        <v>0.7863583520348563</v>
       </c>
       <c r="R46">
-        <v>0.163354111825473</v>
+        <v>0.5989650766934009</v>
       </c>
       <c r="S46">
-        <v>0.130081403451796</v>
+        <v>0.4769651459899187</v>
       </c>
       <c r="T46">
-        <v>0.0864364</v>
+        <v>0.3169334666666667</v>
       </c>
     </row>
     <row r="47" spans="1:20">
@@ -3162,43 +3162,43 @@
         <v>58</v>
       </c>
       <c r="H47">
-        <v>0.00282409</v>
+        <v>0.01035499666666667</v>
       </c>
       <c r="I47">
-        <v>0.034400700109519</v>
+        <v>0.1261359004015697</v>
       </c>
       <c r="J47">
-        <v>0.34330130228</v>
+        <v>1.258771441693333</v>
       </c>
       <c r="K47">
-        <v>0.6233930986352</v>
+        <v>2.285774694995733</v>
       </c>
       <c r="L47">
-        <v>0.8879670750351001</v>
+        <v>3.2558792751287</v>
       </c>
       <c r="M47">
-        <v>1.1388530770129</v>
+        <v>4.175794615713967</v>
       </c>
       <c r="N47">
-        <v>1.375640144727</v>
+        <v>5.044013863998999</v>
       </c>
       <c r="O47">
-        <v>1.613500905674</v>
+        <v>5.916169987471332</v>
       </c>
       <c r="P47">
-        <v>1.82381428129</v>
+        <v>6.687319031396666</v>
       </c>
       <c r="Q47">
-        <v>1.999607954965</v>
+        <v>7.331895834871667</v>
       </c>
       <c r="R47">
-        <v>2.128134852555</v>
+        <v>7.803161126035</v>
       </c>
       <c r="S47">
-        <v>2.242646068886</v>
+        <v>8.223035585915333</v>
       </c>
       <c r="T47">
-        <v>2.2889666176339</v>
+        <v>8.392877597990966</v>
       </c>
     </row>
     <row r="48" spans="1:20">
@@ -3218,40 +3218,40 @@
         <v>58</v>
       </c>
       <c r="F48">
-        <v>9.367252E-07</v>
+        <v>3.434659066666666E-06</v>
       </c>
       <c r="G48">
-        <v>3.3694797E-06</v>
+        <v>1.23547589E-05</v>
       </c>
       <c r="H48">
-        <v>0.00031182051</v>
+        <v>0.00114334187</v>
       </c>
       <c r="I48">
-        <v>0.00025865336</v>
+        <v>0.0009483956533333332</v>
       </c>
       <c r="J48">
-        <v>0.00015636093</v>
+        <v>0.00057332341</v>
       </c>
       <c r="K48">
-        <v>3.0409344E-05</v>
+        <v>0.000111500928</v>
       </c>
       <c r="L48">
-        <v>9.366017E-06</v>
+        <v>3.434206233333334E-05</v>
       </c>
       <c r="M48">
-        <v>4.007071999999999E-06</v>
+        <v>1.469259733333333E-05</v>
       </c>
       <c r="N48">
-        <v>1.9158085E-06</v>
+        <v>7.024631166666667E-06</v>
       </c>
       <c r="O48">
-        <v>1.1286396E-06</v>
+        <v>4.1383452E-06</v>
       </c>
       <c r="P48">
-        <v>7.04296E-07</v>
+        <v>2.582418666666667E-06</v>
       </c>
       <c r="Q48">
-        <v>3.435701E-07</v>
+        <v>1.259757033333333E-06</v>
       </c>
     </row>
     <row r="49" spans="1:20">
@@ -3271,40 +3271,40 @@
         <v>58</v>
       </c>
       <c r="F49">
-        <v>1.21808E-08</v>
+        <v>4.466293333333334E-08</v>
       </c>
       <c r="G49">
-        <v>1.1661E-07</v>
+        <v>4.2757E-07</v>
       </c>
       <c r="H49">
-        <v>9.733E-06</v>
+        <v>3.568766666666667E-05</v>
       </c>
       <c r="I49">
-        <v>3.73197E-05</v>
+        <v>0.0001368389</v>
       </c>
       <c r="J49">
-        <v>0.000120568</v>
+        <v>0.0004420826666666666</v>
       </c>
       <c r="K49">
-        <v>3.25289E-05</v>
+        <v>0.0001192726333333333</v>
       </c>
       <c r="L49">
-        <v>1.32712E-05</v>
+        <v>4.866106666666666E-05</v>
       </c>
       <c r="M49">
-        <v>7.26431E-06</v>
+        <v>2.663580333333333E-05</v>
       </c>
       <c r="N49">
-        <v>4.45345E-06</v>
+        <v>1.632931666666667E-05</v>
       </c>
       <c r="O49">
-        <v>3.25373E-06</v>
+        <v>1.193034333333333E-05</v>
       </c>
       <c r="P49">
-        <v>2.55403E-06</v>
+        <v>9.364776666666668E-06</v>
       </c>
       <c r="Q49">
-        <v>1.5558E-06</v>
+        <v>5.7046E-06</v>
       </c>
     </row>
     <row r="50" spans="1:20">
@@ -3324,49 +3324,49 @@
         <v>58</v>
       </c>
       <c r="F50">
-        <v>3.72482067E-05</v>
+        <v>0.0001365767579</v>
       </c>
       <c r="G50">
-        <v>0.000137299745</v>
+        <v>0.0005034323983333334</v>
       </c>
       <c r="H50">
-        <v>0.029875129886418</v>
+        <v>0.109542142916866</v>
       </c>
       <c r="I50">
-        <v>0.06448233716248</v>
+        <v>0.2364352362624267</v>
       </c>
       <c r="J50">
-        <v>0.16544031193462</v>
+        <v>0.6066144770936066</v>
       </c>
       <c r="K50">
-        <v>0.137015385623876</v>
+        <v>0.5023897472875453</v>
       </c>
       <c r="L50">
-        <v>0.142182531607653</v>
+        <v>0.5213359492280609</v>
       </c>
       <c r="M50">
-        <v>0.1658597109338899</v>
+        <v>0.6081522734242629</v>
       </c>
       <c r="N50">
-        <v>0.203958013534679</v>
+        <v>0.7478460496271564</v>
       </c>
       <c r="O50">
-        <v>0.5781412974047649</v>
+        <v>2.119851423817471</v>
       </c>
       <c r="P50">
-        <v>1.24504916214803</v>
+        <v>4.565180261209443</v>
       </c>
       <c r="Q50">
-        <v>1.52158697311542</v>
+        <v>5.579152234756541</v>
       </c>
       <c r="R50">
-        <v>1.829882996348317</v>
+        <v>6.709570986610497</v>
       </c>
       <c r="S50">
-        <v>2.142533613478438</v>
+        <v>7.855956582754273</v>
       </c>
       <c r="T50">
-        <v>2.47805372539799</v>
+        <v>9.086196993125963</v>
       </c>
     </row>
     <row r="51" spans="1:20">
@@ -3386,49 +3386,49 @@
         <v>58</v>
       </c>
       <c r="F51">
-        <v>5.82487E-08</v>
+        <v>2.135785666666666E-07</v>
       </c>
       <c r="G51">
-        <v>7.9103E-07</v>
+        <v>2.900443333333333E-06</v>
       </c>
       <c r="H51">
-        <v>0.00058525</v>
+        <v>0.002145916666666667</v>
       </c>
       <c r="I51">
-        <v>0.00629447</v>
+        <v>0.02307972333333333</v>
       </c>
       <c r="J51">
-        <v>0.0743707</v>
+        <v>0.2726925666666667</v>
       </c>
       <c r="K51">
-        <v>0.073840585025</v>
+        <v>0.2707488117583334</v>
       </c>
       <c r="L51">
-        <v>0.099758517</v>
+        <v>0.365781229</v>
       </c>
       <c r="M51">
-        <v>0.365096800553333</v>
+        <v>1.338688268695554</v>
       </c>
       <c r="N51">
-        <v>0.556236014101</v>
+        <v>2.039532051703667</v>
       </c>
       <c r="O51">
-        <v>0.8660047399999999</v>
+        <v>3.175350713333333</v>
       </c>
       <c r="P51">
-        <v>1.31291687360162</v>
+        <v>4.814028536539273</v>
       </c>
       <c r="Q51">
-        <v>2.057761884</v>
+        <v>7.545126908</v>
       </c>
       <c r="R51">
-        <v>3.3809078502865</v>
+        <v>12.39666211771716</v>
       </c>
       <c r="S51">
-        <v>5.4386786403</v>
+        <v>19.9418216811</v>
       </c>
       <c r="T51">
-        <v>8.249098231</v>
+        <v>30.24669351366667</v>
       </c>
     </row>
     <row r="52" spans="1:20">
@@ -3448,49 +3448,49 @@
         <v>58</v>
       </c>
       <c r="F52">
-        <v>0.00019524021</v>
+        <v>0.0007158807700000001</v>
       </c>
       <c r="G52">
-        <v>0.0009065484</v>
+        <v>0.003324010799999999</v>
       </c>
       <c r="H52">
-        <v>0.240544644</v>
+        <v>0.8819970279999999</v>
       </c>
       <c r="I52">
-        <v>0.890318179</v>
+        <v>3.264499989666667</v>
       </c>
       <c r="J52">
-        <v>2.6218696270749</v>
+        <v>9.613521965941301</v>
       </c>
       <c r="K52">
-        <v>3.938047343376948</v>
+        <v>14.43950692571548</v>
       </c>
       <c r="L52">
-        <v>5.376977171480006</v>
+        <v>19.71558296209336</v>
       </c>
       <c r="M52">
-        <v>7.052829594897145</v>
+        <v>25.86037518128953</v>
       </c>
       <c r="N52">
-        <v>9.179696863540626</v>
+        <v>33.65888849964896</v>
       </c>
       <c r="O52">
-        <v>12.2301922764568</v>
+        <v>44.84403834700827</v>
       </c>
       <c r="P52">
-        <v>16.268054434612</v>
+        <v>59.64953292691067</v>
       </c>
       <c r="Q52">
-        <v>22.80587841677639</v>
+        <v>83.62155419484678</v>
       </c>
       <c r="R52">
-        <v>29.712851522288</v>
+        <v>108.9471222483893</v>
       </c>
       <c r="S52">
-        <v>38.16887519182701</v>
+        <v>139.9525423700323</v>
       </c>
       <c r="T52">
-        <v>45.9080988868269</v>
+        <v>168.3296959183653</v>
       </c>
     </row>
     <row r="53" spans="1:20">
@@ -3510,49 +3510,49 @@
         <v>58</v>
       </c>
       <c r="F53">
-        <v>1.23883E-06</v>
+        <v>4.542376666666667E-06</v>
       </c>
       <c r="G53">
-        <v>1.82886E-05</v>
+        <v>6.705819999999999E-05</v>
       </c>
       <c r="H53">
-        <v>0.014204538384</v>
+        <v>0.052083307408</v>
       </c>
       <c r="I53">
-        <v>0.1372718</v>
+        <v>0.5033299333333333</v>
       </c>
       <c r="J53">
-        <v>1.1685842752</v>
+        <v>4.284809009066667</v>
       </c>
       <c r="K53">
-        <v>2.06845716604</v>
+        <v>7.584342942146667</v>
       </c>
       <c r="L53">
-        <v>3.0502878654</v>
+        <v>11.1843888398</v>
       </c>
       <c r="M53">
-        <v>4.30445933</v>
+        <v>15.78301754333333</v>
       </c>
       <c r="N53">
-        <v>6.0241007024459</v>
+        <v>22.08836924230163</v>
       </c>
       <c r="O53">
-        <v>8.73778308742</v>
+        <v>32.03853798720667</v>
       </c>
       <c r="P53">
-        <v>12.747619838472</v>
+        <v>46.74127274106399</v>
       </c>
       <c r="Q53">
-        <v>18.59541855202231</v>
+        <v>68.18320135741511</v>
       </c>
       <c r="R53">
-        <v>26.48992303948</v>
+        <v>97.12971781142666</v>
       </c>
       <c r="S53">
-        <v>36.73100304</v>
+        <v>134.68034448</v>
       </c>
       <c r="T53">
-        <v>47.61504281</v>
+        <v>174.5884903033333</v>
       </c>
     </row>
     <row r="54" spans="1:20">
@@ -3572,28 +3572,28 @@
         <v>58</v>
       </c>
       <c r="H54">
-        <v>0.00062989986</v>
+        <v>0.00230963282</v>
       </c>
       <c r="I54">
-        <v>0.0015051872</v>
+        <v>0.005519019733333333</v>
       </c>
       <c r="J54">
-        <v>0.0011692705</v>
+        <v>0.004287325166666666</v>
       </c>
       <c r="K54">
-        <v>0.00018650887</v>
+        <v>0.0006838658566666667</v>
       </c>
       <c r="L54">
-        <v>3.665887E-05</v>
+        <v>0.0001344158566666667</v>
       </c>
       <c r="M54">
-        <v>8.811594000000001E-06</v>
+        <v>3.2309178E-05</v>
       </c>
       <c r="N54">
-        <v>2.234712E-06</v>
+        <v>8.193944E-06</v>
       </c>
       <c r="O54">
-        <v>6.72648E-07</v>
+        <v>2.466376E-06</v>
       </c>
     </row>
     <row r="55" spans="1:20">
@@ -3613,31 +3613,31 @@
         <v>58</v>
       </c>
       <c r="H55">
-        <v>3.86371E-05</v>
+        <v>0.0001416693666666667</v>
       </c>
       <c r="I55">
-        <v>0.000316189</v>
+        <v>0.001159359666666667</v>
       </c>
       <c r="J55">
-        <v>0.00106102</v>
+        <v>0.003890406666666667</v>
       </c>
       <c r="K55">
-        <v>0.00023886</v>
+        <v>0.0008758199999999999</v>
       </c>
       <c r="L55">
-        <v>6.70282E-05</v>
+        <v>0.0002457700666666667</v>
       </c>
       <c r="M55">
-        <v>2.26159E-05</v>
+        <v>8.292496666666668E-05</v>
       </c>
       <c r="N55">
-        <v>8.17868E-06</v>
+        <v>2.998849333333333E-05</v>
       </c>
       <c r="O55">
-        <v>3.46655E-06</v>
+        <v>1.271068333333333E-05</v>
       </c>
       <c r="P55">
-        <v>2.75664E-10</v>
+        <v>1.010768E-09</v>
       </c>
     </row>
     <row r="56" spans="1:20">
@@ -3657,43 +3657,43 @@
         <v>58</v>
       </c>
       <c r="H56">
-        <v>0.024289903</v>
+        <v>0.08906297766666668</v>
       </c>
       <c r="I56">
-        <v>0.08641078568379999</v>
+        <v>0.3168395475072667</v>
       </c>
       <c r="J56">
-        <v>0.199000345055396</v>
+        <v>0.7296679318697855</v>
       </c>
       <c r="K56">
-        <v>0.09712499170745401</v>
+        <v>0.356124969593998</v>
       </c>
       <c r="L56">
-        <v>0.04366304</v>
+        <v>0.1600978133333333</v>
       </c>
       <c r="M56">
-        <v>0.022691513</v>
+        <v>0.08320221433333333</v>
       </c>
       <c r="N56">
-        <v>0.012645477</v>
+        <v>0.04636674899999999</v>
       </c>
       <c r="O56">
-        <v>0.008228062</v>
+        <v>0.03016956066666667</v>
       </c>
       <c r="P56">
-        <v>0.005101497</v>
+        <v>0.018705489</v>
       </c>
       <c r="Q56">
-        <v>0.003285443</v>
+        <v>0.01204662433333334</v>
       </c>
       <c r="R56">
-        <v>0.002104551</v>
+        <v>0.007716687</v>
       </c>
       <c r="S56">
-        <v>0.00159145</v>
+        <v>0.005835316666666666</v>
       </c>
       <c r="T56">
-        <v>0.0009330899999999999</v>
+        <v>0.00342133</v>
       </c>
     </row>
     <row r="57" spans="1:20">
@@ -3713,43 +3713,43 @@
         <v>58</v>
       </c>
       <c r="H57">
-        <v>0.00111292</v>
+        <v>0.004080706666666667</v>
       </c>
       <c r="I57">
-        <v>0.0122265</v>
+        <v>0.0448305</v>
       </c>
       <c r="J57">
-        <v>0.104814000351875</v>
+        <v>0.3843180012902083</v>
       </c>
       <c r="K57">
-        <v>0.0631901332205999</v>
+        <v>0.2316971551421996</v>
       </c>
       <c r="L57">
-        <v>0.036317800568365</v>
+        <v>0.1331652687506717</v>
       </c>
       <c r="M57">
-        <v>0.0232942</v>
+        <v>0.08541206666666668</v>
       </c>
       <c r="N57">
-        <v>0.0160559</v>
+        <v>0.05887163333333334</v>
       </c>
       <c r="O57">
-        <v>0.0124141</v>
+        <v>0.04551836666666667</v>
       </c>
       <c r="P57">
-        <v>0.00962292</v>
+        <v>0.03528404</v>
       </c>
       <c r="Q57">
-        <v>0.0077321</v>
+        <v>0.02835103333333333</v>
       </c>
       <c r="R57">
-        <v>0.00622912</v>
+        <v>0.02284010666666667</v>
       </c>
       <c r="S57">
-        <v>0.00561906</v>
+        <v>0.02060322</v>
       </c>
       <c r="T57">
-        <v>0.00432338</v>
+        <v>0.01585239333333333</v>
       </c>
     </row>
     <row r="58" spans="1:20">
@@ -3769,16 +3769,16 @@
         <v>58</v>
       </c>
       <c r="F58">
-        <v>4.4489249E-08</v>
+        <v>1.631272463333333E-07</v>
       </c>
       <c r="G58">
-        <v>1.608264E-07</v>
+        <v>5.896968E-07</v>
       </c>
       <c r="H58">
-        <v>5.2859928E-07</v>
+        <v>1.938197360000001E-06</v>
       </c>
       <c r="I58">
-        <v>8.848616E-09</v>
+        <v>3.244492533333333E-08</v>
       </c>
     </row>
     <row r="59" spans="1:20">
@@ -3798,16 +3798,16 @@
         <v>58</v>
       </c>
       <c r="F59">
-        <v>3.86252E-10</v>
+        <v>1.416257333333333E-09</v>
       </c>
       <c r="G59">
-        <v>4.43906E-09</v>
+        <v>1.627655333333334E-08</v>
       </c>
       <c r="H59">
-        <v>3.81255E-08</v>
+        <v>1.397935E-07</v>
       </c>
       <c r="I59">
-        <v>4.37461E-09</v>
+        <v>1.604023666666667E-08</v>
       </c>
     </row>
     <row r="60" spans="1:20">
@@ -3827,49 +3827,49 @@
         <v>58</v>
       </c>
       <c r="F60">
-        <v>0.00102746075</v>
+        <v>0.003767356083333334</v>
       </c>
       <c r="G60">
-        <v>0.0056858197</v>
+        <v>0.02084800556666666</v>
       </c>
       <c r="H60">
-        <v>0.702098354</v>
+        <v>2.574360631333333</v>
       </c>
       <c r="I60">
-        <v>2.321265394194578</v>
+        <v>8.51130644538012</v>
       </c>
       <c r="J60">
-        <v>6.343653617415351</v>
+        <v>23.26006326385628</v>
       </c>
       <c r="K60">
-        <v>8.432161977708517</v>
+        <v>30.9179272515979</v>
       </c>
       <c r="L60">
-        <v>12.07624105806146</v>
+        <v>44.27955054622535</v>
       </c>
       <c r="M60">
-        <v>16.46992485983901</v>
+        <v>60.38972448607639</v>
       </c>
       <c r="N60">
-        <v>22.5865853263767</v>
+        <v>82.81747953004789</v>
       </c>
       <c r="O60">
-        <v>29.06285211784646</v>
+        <v>106.5637910987704</v>
       </c>
       <c r="P60">
-        <v>35.81458086417375</v>
+        <v>131.3201298353038</v>
       </c>
       <c r="Q60">
-        <v>43.34888414163031</v>
+        <v>158.9459085193111</v>
       </c>
       <c r="R60">
-        <v>50.04871082898104</v>
+        <v>183.5119397062638</v>
       </c>
       <c r="S60">
-        <v>56.54444098712523</v>
+        <v>207.3296169527925</v>
       </c>
       <c r="T60">
-        <v>58.83891559994099</v>
+        <v>215.742690533117</v>
       </c>
     </row>
     <row r="61" spans="1:20">
@@ -3889,49 +3889,49 @@
         <v>58</v>
       </c>
       <c r="F61">
-        <v>6.20195E-06</v>
+        <v>2.274048333333333E-05</v>
       </c>
       <c r="G61">
-        <v>9.21356E-05</v>
+        <v>0.0003378305333333333</v>
       </c>
       <c r="H61">
-        <v>0.0252269</v>
+        <v>0.09249863333333334</v>
       </c>
       <c r="I61">
-        <v>0.22704900113623</v>
+        <v>0.8325130041661767</v>
       </c>
       <c r="J61">
-        <v>2.51780294835067</v>
+        <v>9.231944143952457</v>
       </c>
       <c r="K61">
-        <v>4.716645527377126</v>
+        <v>17.29436693371613</v>
       </c>
       <c r="L61">
-        <v>7.038253736961586</v>
+        <v>25.80693036885915</v>
       </c>
       <c r="M61">
-        <v>9.99782900485727</v>
+        <v>36.65870635114332</v>
       </c>
       <c r="N61">
-        <v>13.826159357706</v>
+        <v>50.695917644922</v>
       </c>
       <c r="O61">
-        <v>19.59131609</v>
+        <v>71.83482566333333</v>
       </c>
       <c r="P61">
-        <v>27.54931683209709</v>
+        <v>101.0141617176893</v>
       </c>
       <c r="Q61">
-        <v>38.34029279788</v>
+        <v>140.5810735922267</v>
       </c>
       <c r="R61">
-        <v>50.68580697349</v>
+        <v>185.8479589027967</v>
       </c>
       <c r="S61">
-        <v>63.87668047</v>
+        <v>234.2144950566667</v>
       </c>
       <c r="T61">
-        <v>74.8060665</v>
+        <v>274.2889105</v>
       </c>
     </row>
     <row r="62" spans="1:20">
@@ -3951,43 +3951,43 @@
         <v>58</v>
       </c>
       <c r="H62">
-        <v>0.00130280289</v>
+        <v>0.00477694393</v>
       </c>
       <c r="I62">
-        <v>0.0038668449</v>
+        <v>0.0141784313</v>
       </c>
       <c r="J62">
-        <v>0.008648158600000001</v>
+        <v>0.03170991486666667</v>
       </c>
       <c r="K62">
-        <v>0.0031059629</v>
+        <v>0.01138853063333333</v>
       </c>
       <c r="L62">
-        <v>0.0012640056</v>
+        <v>0.0046346872</v>
       </c>
       <c r="M62">
-        <v>0.0006110714</v>
+        <v>0.002240595133333333</v>
       </c>
       <c r="N62">
-        <v>0.00033453289</v>
+        <v>0.001226620596666667</v>
       </c>
       <c r="O62">
-        <v>0.00020848939</v>
+        <v>0.0007644610966666667</v>
       </c>
       <c r="P62">
-        <v>0.00012599215</v>
+        <v>0.0004619712166666667</v>
       </c>
       <c r="Q62">
-        <v>8.153795E-05</v>
+        <v>0.0002989724833333334</v>
       </c>
       <c r="R62">
-        <v>5.453847E-05</v>
+        <v>0.00019997439</v>
       </c>
       <c r="S62">
-        <v>4.484863E-05</v>
+        <v>0.0001644449766666667</v>
       </c>
       <c r="T62">
-        <v>2.232939E-05</v>
+        <v>8.187443E-05</v>
       </c>
     </row>
     <row r="63" spans="1:20">
@@ -4007,43 +4007,43 @@
         <v>58</v>
       </c>
       <c r="H63">
-        <v>2.62536E-05</v>
+        <v>9.62632E-05</v>
       </c>
       <c r="I63">
-        <v>0.000337069</v>
+        <v>0.001235919666666667</v>
       </c>
       <c r="J63">
-        <v>0.00347502</v>
+        <v>0.01274174</v>
       </c>
       <c r="K63">
-        <v>0.00158415</v>
+        <v>0.00580855</v>
       </c>
       <c r="L63">
-        <v>0.000869116</v>
+        <v>0.003186758666666666</v>
       </c>
       <c r="M63">
-        <v>0.000558678</v>
+        <v>0.002048486</v>
       </c>
       <c r="N63">
-        <v>0.000421311</v>
+        <v>0.001544807</v>
       </c>
       <c r="O63">
-        <v>0.00036852</v>
+        <v>0.00135124</v>
       </c>
       <c r="P63">
-        <v>0.000324929</v>
+        <v>0.001191406333333333</v>
       </c>
       <c r="Q63">
-        <v>0.000293989</v>
+        <v>0.001077959666666667</v>
       </c>
       <c r="R63">
-        <v>0.000272971</v>
+        <v>0.001000893666666667</v>
       </c>
       <c r="S63">
-        <v>0.000276611</v>
+        <v>0.001014240333333333</v>
       </c>
       <c r="T63">
-        <v>0.00021333</v>
+        <v>0.0007822099999999999</v>
       </c>
     </row>
     <row r="64" spans="1:20">
@@ -4063,49 +4063,49 @@
         <v>58</v>
       </c>
       <c r="F64">
-        <v>0.002608253321319</v>
+        <v>0.009563595511503001</v>
       </c>
       <c r="G64">
-        <v>0.012900860729</v>
+        <v>0.04730315600633334</v>
       </c>
       <c r="H64">
-        <v>2.419471896191763</v>
+        <v>8.871396952703131</v>
       </c>
       <c r="I64">
-        <v>8.711017916462398</v>
+        <v>31.94039902702879</v>
       </c>
       <c r="J64">
-        <v>24.67064761016428</v>
+        <v>90.45904123726902</v>
       </c>
       <c r="K64">
-        <v>31.84768141696726</v>
+        <v>116.7748318622133</v>
       </c>
       <c r="L64">
-        <v>41.69686981076967</v>
+        <v>152.8885226394888</v>
       </c>
       <c r="M64">
-        <v>65.15326637263686</v>
+        <v>238.8953100330018</v>
       </c>
       <c r="N64">
-        <v>85.64225943326498</v>
+        <v>314.0216179219716</v>
       </c>
       <c r="O64">
-        <v>110.783241802059</v>
+        <v>406.2052199408828</v>
       </c>
       <c r="P64">
-        <v>139.8084573344035</v>
+        <v>512.6310102261463</v>
       </c>
       <c r="Q64">
-        <v>175.9598238412833</v>
+        <v>645.1860207513722</v>
       </c>
       <c r="R64">
-        <v>216.1137600413759</v>
+        <v>792.4171201517117</v>
       </c>
       <c r="S64">
-        <v>258.8299124601748</v>
+        <v>949.0430123539743</v>
       </c>
       <c r="T64">
-        <v>291.480410800064</v>
+        <v>1068.761506266901</v>
       </c>
     </row>
     <row r="65" spans="1:20">
@@ -4125,49 +4125,49 @@
         <v>58</v>
       </c>
       <c r="F65">
-        <v>1.4801086912E-05</v>
+        <v>5.427065201066667E-05</v>
       </c>
       <c r="G65">
-        <v>0.00021453774226</v>
+        <v>0.0007866383882866666</v>
       </c>
       <c r="H65">
-        <v>0.1046978208095</v>
+        <v>0.3838920096348333</v>
       </c>
       <c r="I65">
-        <v>1.0386554245037</v>
+        <v>3.808403223180233</v>
       </c>
       <c r="J65">
-        <v>10.75700733648593</v>
+        <v>39.44236023378175</v>
       </c>
       <c r="K65">
-        <v>19.13627295025191</v>
+        <v>70.16633415092366</v>
       </c>
       <c r="L65">
-        <v>28.13340537418544</v>
+        <v>103.1558197053466</v>
       </c>
       <c r="M65">
-        <v>39.53553291177946</v>
+        <v>144.9636206765247</v>
       </c>
       <c r="N65">
-        <v>53.82025191860367</v>
+        <v>197.3409237015468</v>
       </c>
       <c r="O65">
-        <v>75.95682378009487</v>
+        <v>278.5083538603478</v>
       </c>
       <c r="P65">
-        <v>106.8368486951606</v>
+        <v>391.7351118822556</v>
       </c>
       <c r="Q65">
-        <v>150.1369967719003</v>
+        <v>550.502321496968</v>
       </c>
       <c r="R65">
-        <v>205.9915930095471</v>
+        <v>755.3025077016728</v>
       </c>
       <c r="S65">
-        <v>276.269284143089</v>
+        <v>1012.987375191326</v>
       </c>
       <c r="T65">
-        <v>350.2389073516671</v>
+        <v>1284.209326956113</v>
       </c>
     </row>
     <row r="66" spans="1:20">

</xml_diff>